<commit_message>
fix(consulting): block bank/equip FPs and regenerate clean RC v2
Reject financial-institution credenciamento/arrecadação and pure equipment
purchases (airless, motobombas) as non-engineering; re-freeze C without
those rows; keep PENDING_HUMAN for second human product review.
</commit_message>
<xml_diff>
--- a/artifacts/campaigns/CLIENT-READY-RECURRING-CONSULTING-CYCLE-01/client-ready-frozen-rc-v2/consulting-pack.xlsx
+++ b/artifacts/campaigns/CLIENT-READY-RECURRING-CONSULTING-CYCLE-01/client-ready-frozen-rc-v2/consulting-pack.xlsx
@@ -642,7 +642,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Status RC: PENDING_HUMAN | Pack: live-pack-20260725-032739-85524edc</t>
+          <t>Status RC: PENDING_HUMAN | Pack: live-pack-20260725-033723-8b07813e</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23">
@@ -1363,16 +1363,16 @@
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>R$ 34.564.663,05</t>
+          <t>R$ 29.626.854,05</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>R$ 735.418,36</t>
+          <t>R$ 740.671,35</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -2161,12 +2161,12 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE MELEIRO - SC</t>
+          <t>Secretário de Infraestrutura</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>82.837.741/0001-96</t>
+          <t>83.102.574/0001-06</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -2175,21 +2175,21 @@
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>R$ 6.093.831,66</t>
+          <t>R$ 19.652.917,97</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>R$ 304.691,58</t>
+          <t>R$ 517.182,05</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>infraestrutura_urbana, obras_civis, pavimentacao, terraplenagem</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
@@ -2197,11 +2197,7 @@
           <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
         </is>
       </c>
-      <c r="J24" s="6" t="inlineStr">
-        <is>
-          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
-        </is>
-      </c>
+      <c r="J24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n">
@@ -2209,12 +2205,12 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Secretário de Infraestrutura</t>
+          <t>PREFEITURA MUNICIPAL DE XAXIM - SC</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>83.102.574/0001-06</t>
+          <t>82.854.670/0001-30</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2223,21 +2219,21 @@
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>R$ 19.652.917,97</t>
+          <t>R$ 17.730.435,59</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>R$ 517.182,05</t>
+          <t>R$ 985.024,20</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>infraestrutura_urbana, pavimentacao</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
@@ -2245,7 +2241,11 @@
           <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
         </is>
       </c>
-      <c r="J25" s="6" t="inlineStr"/>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n">
@@ -2253,12 +2253,12 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE XAXIM - SC</t>
+          <t>PREFEITURA MUNICIPAL DE NOVA TRENTO</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>82.854.670/0001-30</t>
+          <t>82.925.025/0001-60</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -2267,21 +2267,21 @@
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>R$ 17.730.435,59</t>
+          <t>R$ 27.535.493,77</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>R$ 985.024,20</t>
+          <t>R$ 949.499,79</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>infraestrutura_urbana, pavimentacao</t>
+          <t>obras_civis, pavimentacao</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -2301,12 +2301,12 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE NOVA TRENTO</t>
+          <t>PREFEITURA MUNICIPAL DE TREZE DE MAIO - SC</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>82.925.025/0001-60</t>
+          <t>82.928.672/0001-26</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -2315,21 +2315,21 @@
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>R$ 27.535.493,77</t>
+          <t>R$ 16.416.747,77</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>R$ 949.499,79</t>
+          <t>R$ 713.771,64</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>obras_civis, pavimentacao</t>
+          <t>manutencao_predial, obras_civis, pavimentacao</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -2349,12 +2349,12 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE TREZE DE MAIO - SC</t>
+          <t>SECRETARIA DE OBRAS E TRANSPORTES</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>82.928.672/0001-26</t>
+          <t>82.915.232/0001-34</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -2363,21 +2363,21 @@
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>R$ 16.416.747,77</t>
+          <t>R$ 18.819.602,95</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>R$ 713.771,64</t>
+          <t>R$ 672.128,68</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>manutencao_predial, obras_civis, pavimentacao</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
@@ -2397,12 +2397,12 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>SECRETARIA DE OBRAS E TRANSPORTES</t>
+          <t>MOBILIDADE URBANA</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>82.915.232/0001-34</t>
+          <t>86.051.398/0001-00</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -2411,16 +2411,16 @@
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>R$ 18.819.602,95</t>
+          <t>R$ 46.132.091,18</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>R$ 672.128,68</t>
+          <t>R$ 2.096.913,24</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
@@ -2445,12 +2445,12 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Secretaria de Administração</t>
+          <t>PREFEITURA MUNICIPAL DE PALMITOS - SC</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>83.102.228/0001-10</t>
+          <t>85.361.863/0001-47</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2459,21 +2459,21 @@
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>R$ 10.253.157,38</t>
+          <t>R$ 31.739.938,05</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>R$ 394.352,21</t>
+          <t>R$ 1.322.497,42</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>infraestrutura_urbana, pavimentacao</t>
+          <t>infraestrutura_urbana, pavimentacao, terraplenagem</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
@@ -2493,12 +2493,12 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>MOBILIDADE URBANA</t>
+          <t>MUNICÍPIO DE SANTO AMARO DA IMPERATRIZ</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>86.051.398/0001-00</t>
+          <t>82.892.324/0001-46</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -2507,21 +2507,21 @@
         </is>
       </c>
       <c r="E31" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>R$ 46.132.091,18</t>
+          <t>R$ 9.506.607,04</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>R$ 2.096.913,24</t>
+          <t>R$ 594.162,94</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>obras_civis, pavimentacao</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
@@ -2541,12 +2541,12 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE PALMITOS - SC</t>
+          <t>SECRETARIA MUNICIPAL DE INFRA ESTRUTURA</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>85.361.863/0001-47</t>
+          <t>82.926.569/0001-47</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -2555,21 +2555,21 @@
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>R$ 31.739.938,05</t>
+          <t>R$ 12.789.758,10</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>R$ 1.322.497,42</t>
+          <t>R$ 412.572,84</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>infraestrutura_urbana, pavimentacao, terraplenagem</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -2577,11 +2577,7 @@
           <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
         </is>
       </c>
-      <c r="J32" s="6" t="inlineStr">
-        <is>
-          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
-        </is>
-      </c>
+      <c r="J32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
@@ -2589,12 +2585,12 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>MUNICÍPIO DE SANTO AMARO DA IMPERATRIZ</t>
+          <t>Departamento de Obras Públicas</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>82.892.324/0001-46</t>
+          <t>81.140.303/0001-01</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -2603,21 +2599,21 @@
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>R$ 9.506.607,04</t>
+          <t>R$ 21.063.138,66</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>R$ 594.162,94</t>
+          <t>R$ 957.415,39</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>obras_civis, pavimentacao</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -2637,12 +2633,12 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>SECRETARIA MUNICIPAL DE INFRA ESTRUTURA</t>
+          <t>PREFEITURA MUNICIPAL DE CORDILHEIRA ALTA - SC</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>82.926.569/0001-47</t>
+          <t>95.990.198/0001-04</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -2651,21 +2647,21 @@
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>R$ 12.789.758,10</t>
+          <t>R$ 7.153.590,03</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>R$ 412.572,84</t>
+          <t>R$ 376.504,74</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>obras_civis, pavimentacao, saneamento</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
@@ -2673,7 +2669,11 @@
           <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
         </is>
       </c>
-      <c r="J34" s="6" t="inlineStr"/>
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
@@ -2681,12 +2681,12 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Departamento de Obras Públicas</t>
+          <t>Prefeitura de Gaspar - SC</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>81.140.303/0001-01</t>
+          <t>83.102.244/0001-02</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -2695,16 +2695,16 @@
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>R$ 21.063.138,66</t>
+          <t>R$ 28.777.208,92</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>R$ 957.415,39</t>
+          <t>R$ 1.798.575,56</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
@@ -2729,12 +2729,12 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE CORDILHEIRA ALTA - SC</t>
+          <t>SECRETARIA MUNICIPAL DE OBRAS E PLANEJAMENTO</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>95.990.198/0001-04</t>
+          <t>83.102.319/0001-55</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -2743,21 +2743,21 @@
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>R$ 7.153.590,03</t>
+          <t>R$ 17.884.066,11</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>R$ 376.504,74</t>
+          <t>R$ 851.622,20</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>obras_civis, pavimentacao, saneamento</t>
+          <t>drenagem, obras_civis, pavimentacao</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
@@ -2777,12 +2777,12 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Prefeitura de Gaspar - SC</t>
+          <t>MUNICÍPIO DE ORLEANS</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>83.102.244/0001-02</t>
+          <t>82.926.544/0001-43</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -2791,21 +2791,21 @@
         </is>
       </c>
       <c r="E37" s="6" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>R$ 28.777.208,92</t>
+          <t>R$ 18.131.060,72</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>R$ 1.798.575,56</t>
+          <t>R$ 788.306,99</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>obras_civis, pavimentacao, terraplenagem</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
@@ -2825,12 +2825,12 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>SECRETARIA MUNICIPAL DE OBRAS E PLANEJAMENTO</t>
+          <t>Departamento de Urbanismo</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>83.102.319/0001-55</t>
+          <t>83.102.640/0001-30</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -2839,21 +2839,21 @@
         </is>
       </c>
       <c r="E38" s="6" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>R$ 17.884.066,11</t>
+          <t>R$ 18.723.510,96</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>R$ 851.622,20</t>
+          <t>R$ 668.696,82</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>drenagem, obras_civis, pavimentacao</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
@@ -2861,11 +2861,7 @@
           <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
         </is>
       </c>
-      <c r="J38" s="6" t="inlineStr">
-        <is>
-          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
-        </is>
-      </c>
+      <c r="J38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n">
@@ -2873,12 +2869,12 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>MUNICÍPIO DE ORLEANS</t>
+          <t>Câmara de Vereadores de Balneário Camboriú</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>82.926.544/0001-43</t>
+          <t>83.551.549/0001-00</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -2887,21 +2883,21 @@
         </is>
       </c>
       <c r="E39" s="6" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>R$ 18.131.060,72</t>
+          <t>R$ 466.924,14</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>R$ 788.306,99</t>
+          <t>R$ 31.128,28</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>obras_civis, pavimentacao, terraplenagem</t>
+          <t>manutencao_predial, obras_civis</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -2921,12 +2917,12 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Departamento de Urbanismo</t>
+          <t>PREFEITURA MUNICIPAL DE HERVAL D´OESTE - SC</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>83.102.640/0001-30</t>
+          <t>82.939.430/0001-38</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -2935,21 +2931,21 @@
         </is>
       </c>
       <c r="E40" s="6" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>R$ 18.723.510,96</t>
+          <t>R$ 21.086.567,78</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>R$ 668.696,82</t>
+          <t>R$ 958.480,35</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>infraestrutura_urbana, pavimentacao</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
@@ -2957,7 +2953,11 @@
           <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
         </is>
       </c>
-      <c r="J40" s="6" t="inlineStr"/>
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
@@ -2965,12 +2965,12 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Câmara de Vereadores de Balneário Camboriú</t>
+          <t>MUNICÍPIO DE LAURO MULLER</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>83.551.549/0001-00</t>
+          <t>82.558.909/0001-24</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -2979,21 +2979,21 @@
         </is>
       </c>
       <c r="E41" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>R$ 466.924,14</t>
+          <t>R$ 8.786.664,76</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>R$ 31.128,28</t>
+          <t>R$ 675.897,29</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>manutencao_predial, obras_civis</t>
+          <t>obras_civis, pavimentacao, terraplenagem</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
@@ -4725,22 +4725,22 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Serviço Autônomo Municipal de Agua e Esgoto- Blumenau SC</t>
+          <t>Departamento de Turismo</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>CREDENCIAMENTO DE INSTITUIÇÕES FINANCEIRAS DEVIDAMENTE AUTORIZADAS A OPERAR PELO BANCO CENTRAL DO BRASIL, NAS MODALIDADES DE BANCO MÚLTIPLO, BANCO COMERCIAL, BANCO COOPERATIVO OU COOPERATIVA DE CRÉDITO, COM A FINALIDADE DE EXECUTAR SERVIÇOS DE ARRECADAÇÃO DE FATURAS REFERENTES AO FORNECIMENTO DE ÁGUA, ESGOTAMENTO SANITÁRIO, COLETA DE RESÍDUOS SÓLIDOS, BEM COMO DA DÍVIDA ATIVA E DEMAIS RECEITAS SOB A RESPONSABILIDADE DESTA AUTARQUIA.</t>
+          <t>Contratação de empresa especializada no ramo da construção civil, em regime de empreitada por preço unitário, com fornecimento de materiais e mão de obra, para execução de serviços referentes a construção de edificação destinada ao quiosque na Prainha de Linha Bonita, Município de Itá/SC.</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>BANCO COOPERATIVO SICOOB S/A</t>
+          <t>ECGT CONSTRUCOES LTDA</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>02.038.232/0001-64</t>
+          <t>06.907.152/0001-59</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -4750,12 +4750,12 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>R$ 342.000,00</t>
+          <t>R$ 332.500,00</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>saneamento</t>
+          <t>edificacoes</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -4782,22 +4782,22 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Departamento de Turismo</t>
+          <t>SECRETARIA DE ADMINISTRAÇÃO E FINANÇAS</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada no ramo da construção civil, em regime de empreitada por preço unitário, com fornecimento de materiais e mão de obra, para execução de serviços referentes a construção de edificação destinada ao quiosque na Prainha de Linha Bonita, Município de Itá/SC.</t>
+          <t>REF.: O PRESENTE PROCEDIMENTO LICITATÓRIO TEM POR OBJETIVO SELECIONAR A PROPOSTA MAIS VANTAJOSA PARA FUTURA E EVENTUAL A CONTRATAÇÃO DE EMPRESA DE ENGENHARIA ESPECIALIZADA PARA EXECUÇÃO DA REFORMA E REVITALIZAÇÃO DO CEMITÉRIO NA COMUNIDADE DE VILA SÃO CRISTÓVÃO, MUNICÍPIO DE SANTA ROSA DO SUL/SC, CONFORME AS ESPECIFICAÇÕES CONSTANTES NO EDITAL, CRONOGRAMA FÍSICO-FINANCEIRO, MEMORIAL DESCRITIVO, PLANILHA ORÇAMENTÁRIA, PROJETO E DEMAIS ANEXOS. (TE 0091/2026)</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>ECGT CONSTRUCOES LTDA</t>
+          <t>SUDOESTE CONSTRUÇÕES LTDA</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>06.907.152/0001-59</t>
+          <t>64.767.020/0001-75</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -4807,12 +4807,12 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>R$ 332.500,00</t>
+          <t>R$ 200.000,00</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>edificacoes</t>
+          <t>infraestrutura_urbana</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -4839,22 +4839,22 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ADMINISTRAÇÃO E FINANÇAS</t>
+          <t>Diretoria do Arquivo Público</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>REF.: O PRESENTE PROCEDIMENTO LICITATÓRIO TEM POR OBJETIVO SELECIONAR A PROPOSTA MAIS VANTAJOSA PARA FUTURA E EVENTUAL A CONTRATAÇÃO DE EMPRESA DE ENGENHARIA ESPECIALIZADA PARA EXECUÇÃO DA REFORMA E REVITALIZAÇÃO DO CEMITÉRIO NA COMUNIDADE DE VILA SÃO CRISTÓVÃO, MUNICÍPIO DE SANTA ROSA DO SUL/SC, CONFORME AS ESPECIFICAÇÕES CONSTANTES NO EDITAL, CRONOGRAMA FÍSICO-FINANCEIRO, MEMORIAL DESCRITIVO, PLANILHA ORÇAMENTÁRIA, PROJETO E DEMAIS ANEXOS. (TE 0091/2026)</t>
+          <t>Contratação  de serviços de engenharia para  execução  de manutenção predial corretiva e preventiva (via ARP 201/2025) para imóvel SIGEP 4765, sede administrativa da CODAM Criciúma, localizada na Rua José de Patta, 120, Centro, Criciúma/SC.</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>SUDOESTE CONSTRUÇÕES LTDA</t>
+          <t>AEJ ENGENHARIA LTDA</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>64.767.020/0001-75</t>
+          <t>54.960.587/0001-00</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -4864,12 +4864,12 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>R$ 200.000,00</t>
+          <t>R$ 139.084,03</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>infraestrutura_urbana</t>
+          <t>obras_civis</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -4896,7 +4896,7 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Diretoria do Arquivo Público</t>
+          <t>Instituto do Meio Ambiente do Estado de Santa Catarina</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
@@ -4953,22 +4953,22 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Instituto do Meio Ambiente do Estado de Santa Catarina</t>
+          <t>FUNDO MUNICIPAL DE SAÚDE DE BELMONTE</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Contratação  de serviços de engenharia para  execução  de manutenção predial corretiva e preventiva (via ARP 201/2025) para imóvel SIGEP 4765, sede administrativa da CODAM Criciúma, localizada na Rua José de Patta, 120, Centro, Criciúma/SC.</t>
+          <t>CONTRATAÇÃO DE EMPRESA PARA PRESTAÇÃO DE SERVIÇOS DE MÃO DE OBRA COM FORNECIMENTO DE MATERIAIS PARA EXECUÇÃO DE OBRA DE INFRAESTRUTURA URBANA - PAVIMENTAÇÃO COM PEDRAS IRREGULARES, NO TRECHO DA RUA GENERAL OSÓRIO, COM LARGURA DE RUA DE 15,00 METROS, TOTALIZANDO ÁREA DE 845,53 M², COM LARGURA MÉDIA DE PISTA DE ROLAMENTO DE 10,00 METROS E PASSEIO LATERAL DE 2,50 METROS CADA LADO, COM RECURSOS PRÓPRIOS, DE ACORDO COM OS PROJETOS, MEMORIAL DESCRITIVO, ORÇAMENTOS, CRONOGRAMA FÍSICO FINANCEIRO E DE...</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>AEJ ENGENHARIA LTDA</t>
+          <t>IMPERIAL EMPREENDIMENTOS LTDA</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>54.960.587/0001-00</t>
+          <t>02.645.439/0001-05</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
@@ -4978,12 +4978,12 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>R$ 139.084,03</t>
+          <t>R$ 119.000,00</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>obras_civis</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
@@ -5010,37 +5010,37 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>FUNDO MUNICIPAL DE SAÚDE DE BELMONTE</t>
+          <t>PREFEITURA MUNICIPAL DE IÇARA - SC</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA PARA PRESTAÇÃO DE SERVIÇOS DE MÃO DE OBRA COM FORNECIMENTO DE MATERIAIS PARA EXECUÇÃO DE OBRA DE INFRAESTRUTURA URBANA - PAVIMENTAÇÃO COM PEDRAS IRREGULARES, NO TRECHO DA RUA GENERAL OSÓRIO, COM LARGURA DE RUA DE 15,00 METROS, TOTALIZANDO ÁREA DE 845,53 M², COM LARGURA MÉDIA DE PISTA DE ROLAMENTO DE 10,00 METROS E PASSEIO LATERAL DE 2,50 METROS CADA LADO, COM RECURSOS PRÓPRIOS, DE ACORDO COM OS PROJETOS, MEMORIAL DESCRITIVO, ORÇAMENTOS, CRONOGRAMA FÍSICO FINANCEIRO E DE...</t>
+          <t>CONTRATAÇÃO DE EMPRESA OBJETIVANDO A EXECUÇÃO DA REVITALIZAÇÃO DA PRAÇA FRIDOLINO SCHUEROFF NO BAIRRO PRESIDENTE VARGAS, CONTANDO COM CERCA DE 8.605 M² DE ÁREA CONSTRUÍDA APÓS AMPLIAÇÃO.</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>IMPERIAL EMPREENDIMENTOS LTDA</t>
+          <t>JM PRESTADORA DE SERVIÇOS E CONSTRUÇÃO LTDA</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>02.645.439/0001-05</t>
+          <t>59.022.748/0001-38</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>25/10/2026</t>
+          <t>26/10/2026</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>R$ 119.000,00</t>
+          <t>R$ 115.672,70</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>infraestrutura_urbana</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
@@ -5067,42 +5067,42 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE IÇARA - SC</t>
+          <t>Secretaria Municipal de Planejamento - SEPLAN</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA OBJETIVANDO A EXECUÇÃO DA REVITALIZAÇÃO DA PRAÇA FRIDOLINO SCHUEROFF NO BAIRRO PRESIDENTE VARGAS, CONTANDO COM CERCA DE 8.605 M² DE ÁREA CONSTRUÍDA APÓS AMPLIAÇÃO.</t>
+          <t>Serviços de manutenção predial preventiva, corretiva, bem como reformas prediais sem acréscimo de área construída, abrangendo as áreas civil, elétrica, hidráulica e de sistemas preventivos de combate a incêndio, em todas as unidades administrativas sob responsabilidade do Município de Concórdia.</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>JM PRESTADORA DE SERVIÇOS E CONSTRUÇÃO LTDA</t>
+          <t>CONSTRUTORA FOSCARINI EIRELI</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>59.022.748/0001-38</t>
+          <t>11.517.944/0001-57</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>26/10/2026</t>
+          <t>27/10/2026</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>R$ 115.672,70</t>
+          <t>R$ 3.880.000,00</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>infraestrutura_urbana</t>
+          <t>manutencao_predial</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_HIGH_CONFIDENCE</t>
+          <t>ENGINEERING_REVIEW</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
@@ -5117,29 +5117,29 @@
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_HIGH_CONFIDENCE</t>
+          <t>ENGINEERING_REVIEW</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Secretaria Municipal de Planejamento - SEPLAN</t>
+          <t>PREFEITURA MUNICIPAL DE ITAJAÍ - SC</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Serviços de manutenção predial preventiva, corretiva, bem como reformas prediais sem acréscimo de área construída, abrangendo as áreas civil, elétrica, hidráulica e de sistemas preventivos de combate a incêndio, em todas as unidades administrativas sob responsabilidade do Município de Concórdia.</t>
+          <t>CONTRATAÇÃO DE EMPRESA PARA EXECUÇÃO DAS OBRAS DE PAVIMENTAÇÃO, DRENAGEM PLUVIAL, PASSEIO PÚBLICO E SINALIZAÇÃO VERTICAL NA RUA AUGUSTO CUGNIER</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>CONSTRUTORA FOSCARINI EIRELI</t>
+          <t>C R ARTEFATOS DE CIMENTO LTDA</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>11.517.944/0001-57</t>
+          <t>01.650.178/0001-40</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -5149,17 +5149,17 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>R$ 3.880.000,00</t>
+          <t>R$ 3.269.997,63</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>manutencao_predial</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_REVIEW</t>
+          <t>ENGINEERING_HIGH_CONFIDENCE</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
@@ -5174,29 +5174,29 @@
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_REVIEW</t>
+          <t>ENGINEERING_HIGH_CONFIDENCE</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE ITAJAÍ - SC</t>
+          <t>Serviços Urbanos</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA PARA EXECUÇÃO DAS OBRAS DE PAVIMENTAÇÃO, DRENAGEM PLUVIAL, PASSEIO PÚBLICO E SINALIZAÇÃO VERTICAL NA RUA AUGUSTO CUGNIER</t>
+          <t>Contratação de empresa especializada para a execução de pavimentação em concreto rígido, drenagem pluvial e sinalização viária da Rua Prefeito August Heinrich Purnhagen, localizada no Bairro Universitário, Taió/SC, com extensão de 865,00 metros</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>C R ARTEFATOS DE CIMENTO LTDA</t>
+          <t>MILENIUM SOLUCOES E SERVICOS LTDA</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>01.650.178/0001-40</t>
+          <t>05.594.191/0001-80</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>R$ 3.269.997,63</t>
+          <t>R$ 1.885.100,00</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -5238,22 +5238,22 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Serviços Urbanos</t>
+          <t>DIRETORIA DE TURISMO</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para a execução de pavimentação em concreto rígido, drenagem pluvial e sinalização viária da Rua Prefeito August Heinrich Purnhagen, localizada no Bairro Universitário, Taió/SC, com extensão de 865,00 metros</t>
+          <t>CONTRATAÇÃO DE PESSOA JURÍDICA PARA PRESTAÇÃO DE SERVIÇOS DE ENGENHARIA COM FORNECIMENTO DE MATERIAIS, EQUIPAMENTOS E MÃO DE OBRA PARA CONSTRUÇÃO DE PORTAL DE ENTRADA E REVITALIZAÇÃO DA RUA TRENTO, BAIRRO DIVINÉIA, NO MUNICÍPIO DE RIO DOS CEDROS/SC, EM CONFORMIDADE COM O PROJETO BÁSICO, MEMORIAL DESCRITIVO E DEMAIS ANEXOS DO EDITAL.</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>MILENIUM SOLUCOES E SERVICOS LTDA</t>
+          <t>F9 CONSTRUTORA LTDA</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>05.594.191/0001-80</t>
+          <t>50.032.977/0001-69</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -5263,12 +5263,12 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>R$ 1.885.100,00</t>
+          <t>R$ 753.000,00</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>infraestrutura_urbana</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
@@ -5295,22 +5295,22 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>DIRETORIA DE TURISMO</t>
+          <t>TRIBUNAL REGIONAL DO TRABALHO DA 12A.REGIAO</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE PESSOA JURÍDICA PARA PRESTAÇÃO DE SERVIÇOS DE ENGENHARIA COM FORNECIMENTO DE MATERIAIS, EQUIPAMENTOS E MÃO DE OBRA PARA CONSTRUÇÃO DE PORTAL DE ENTRADA E REVITALIZAÇÃO DA RUA TRENTO, BAIRRO DIVINÉIA, NO MUNICÍPIO DE RIO DOS CEDROS/SC, EM CONFORMIDADE COM O PROJETO BÁSICO, MEMORIAL DESCRITIVO E DEMAIS ANEXOS DO EDITAL.</t>
+          <t>Adequação e reforma do 7º pavimento do prédio sede para instalação de 2 (dois) gabinetes de desembargadores.</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>F9 CONSTRUTORA LTDA</t>
+          <t>LAMINA CONSTRUCOES LTDA</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>50.032.977/0001-69</t>
+          <t>19.534.597/0001-82</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -5320,12 +5320,12 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>R$ 753.000,00</t>
+          <t>R$ 350.987,50</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>infraestrutura_urbana</t>
+          <t>reformas</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
@@ -5352,22 +5352,22 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>TRIBUNAL REGIONAL DO TRABALHO DA 12A.REGIAO</t>
+          <t>Prefeitura Municipal de Chapecó</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Adequação e reforma do 7º pavimento do prédio sede para instalação de 2 (dois) gabinetes de desembargadores.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA EXECUÇÃO DE REVITALIZAÇÃO DA ILUMINAÇÃO DA PONTE ENTRE A DIVISA DE SANTA CATARINA (CHAPECÓ) COM O RIO GRANDE DO SUL (NONOAI).</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>LAMINA CONSTRUCOES LTDA</t>
+          <t>ELETROTEC SISTEMAS DE ENERGIA LTDA</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>19.534.597/0001-82</t>
+          <t>11.796.575/0001-89</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -5377,12 +5377,12 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>R$ 350.987,50</t>
+          <t>R$ 318.000,00</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>reformas</t>
+          <t>infraestrutura_urbana</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
@@ -5409,22 +5409,22 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Prefeitura Municipal de Chapecó</t>
+          <t>SECRETARIA MUNICIPAL DE PLANEJAMENTO E DESENVOLVIMENTO ECONÔMICO SUSTENTÁVEL</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA EXECUÇÃO DE REVITALIZAÇÃO DA ILUMINAÇÃO DA PONTE ENTRE A DIVISA DE SANTA CATARINA (CHAPECÓ) COM O RIO GRANDE DO SUL (NONOAI).</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA A ELABORAÇÃO DE PROJETO DE ENGENHARIA EM NÍVEL EXECUTIVO VISANDO A EXTENSÃO DE VIA ATÉ A PONTE SOBRE O RIO PIÇARRAS, BEM COMO PARA A REALIZAÇÃO DE ESTUDOS, PROGRAMAS, PLANOS E PROJETOS AMBIENTAIS, INCLUINDO COMPLEMENTAÇÕES E ACOMPANHAMENTO DOS PROCESSOS DE LICENCIAMENTO AMBIENTAL.</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>ELETROTEC SISTEMAS DE ENERGIA LTDA</t>
+          <t>GEOMAPA ENGENHARIA LTDA</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>11.796.575/0001-89</t>
+          <t>03.339.646/0001-96</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
@@ -5434,17 +5434,17 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>R$ 318.000,00</t>
+          <t>R$ 163.980,00</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>infraestrutura_urbana</t>
+          <t>projetos</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_HIGH_CONFIDENCE</t>
+          <t>ENGINEERING_REVIEW</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
@@ -5459,29 +5459,29 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_HIGH_CONFIDENCE</t>
+          <t>ENGINEERING_REVIEW</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>SECRETARIA MUNICIPAL DE PLANEJAMENTO E DESENVOLVIMENTO ECONÔMICO SUSTENTÁVEL</t>
+          <t>MUNICÍPIO DE URUBICI</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA A ELABORAÇÃO DE PROJETO DE ENGENHARIA EM NÍVEL EXECUTIVO VISANDO A EXTENSÃO DE VIA ATÉ A PONTE SOBRE O RIO PIÇARRAS, BEM COMO PARA A REALIZAÇÃO DE ESTUDOS, PROGRAMAS, PLANOS E PROJETOS AMBIENTAIS, INCLUINDO COMPLEMENTAÇÕES E ACOMPANHAMENTO DOS PROCESSOS DE LICENCIAMENTO AMBIENTAL.</t>
+          <t>Contratação de empresa especializada para elaboração de projetos técnicos necessários à reforma do salão do CTG – CENTRO DE TRADIÇOES GAÚCHAS - URUBICI contemplando: Projeto Preventivo contra Incêndio (PPCI), projeto hidrossanitário, projeto elétrico, projeto de gás, projeto de climatização, projeto estrutural (área de expansão), com todo acervo necessário, de acordo com o projeto arquitetônico em anexo.</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>GEOMAPA ENGENHARIA LTDA</t>
+          <t>ALTITUDE ENGENHARIA LTDA</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>03.339.646/0001-96</t>
+          <t>42.792.909/0001-70</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
@@ -5491,7 +5491,7 @@
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>R$ 163.980,00</t>
+          <t>R$ 27.000,00</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
@@ -5523,42 +5523,42 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>MUNICÍPIO DE URUBICI</t>
+          <t>SECRETARIA DE INFRAESTRUTURA URBANA</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para elaboração de projetos técnicos necessários à reforma do salão do CTG – CENTRO DE TRADIÇOES GAÚCHAS - URUBICI contemplando: Projeto Preventivo contra Incêndio (PPCI), projeto hidrossanitário, projeto elétrico, projeto de gás, projeto de climatização, projeto estrutural (área de expansão), com todo acervo necessário, de acordo com o projeto arquitetônico em anexo.</t>
+          <t>Contratação de empresa especializada para prestação de serviços de pavimentação de vias urbanas, localizadas junto ao Bairro São Miguel, localizadas nesta cidade de Fraiburgo/SC, conforme especificações deste Termo, Projetos, Memoriais Descritivos e Quantitativos (anexos ao PAL e parte dele integrante):</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>ALTITUDE ENGENHARIA LTDA</t>
+          <t>RA PAVIMENTAÇÕES LTDA</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>42.792.909/0001-70</t>
+          <t>33.062.208/0001-94</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>27/10/2026</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>R$ 27.000,00</t>
+          <t>R$ 2.626.200,00</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>projetos</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_REVIEW</t>
+          <t>ENGINEERING_HIGH_CONFIDENCE</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -5573,29 +5573,29 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_REVIEW</t>
+          <t>ENGINEERING_HIGH_CONFIDENCE</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>SECRETARIA DE INFRAESTRUTURA URBANA</t>
+          <t>Secretaria de Educação, Esporte e Cultura</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para prestação de serviços de pavimentação de vias urbanas, localizadas junto ao Bairro São Miguel, localizadas nesta cidade de Fraiburgo/SC, conforme especificações deste Termo, Projetos, Memoriais Descritivos e Quantitativos (anexos ao PAL e parte dele integrante):</t>
+          <t>CONCORRÊNCIA ELETRÔNICA PARA CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA REALIZAR ASFALTAMENTO DAS RUAS PADRE ADALBERTO ORTHMANN, PADRE FRANZ E ALWIN WEINRICH, LOCALIZADAS NO CENTRO DO MUNICÍPIO DE PRESIDENTE GETÚLIO.</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>RA PAVIMENTAÇÕES LTDA</t>
+          <t>FJ CONSTRUTORA LTDA</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>33.062.208/0001-94</t>
+          <t>27.743.102/0001-53</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
@@ -5605,7 +5605,7 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>R$ 2.626.200,00</t>
+          <t>R$ 1.050.000,00</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -5637,22 +5637,22 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Secretaria de Educação, Esporte e Cultura</t>
+          <t>SECRETARIA DE INFRAESTRUTURA URBANA</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA ELETRÔNICA PARA CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA REALIZAR ASFALTAMENTO DAS RUAS PADRE ADALBERTO ORTHMANN, PADRE FRANZ E ALWIN WEINRICH, LOCALIZADAS NO CENTRO DO MUNICÍPIO DE PRESIDENTE GETÚLIO.</t>
+          <t>Pavimentação em pedras irregulares de basalto nas Ruas "A" Trecho II, "B" Trecho III e "H" no Bairro Nossa Senhora Aparecida.</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>FJ CONSTRUTORA LTDA</t>
+          <t>J.M.A TERRAPLANAGEM LTDA</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>27.743.102/0001-53</t>
+          <t>43.637.217/0001-10</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
@@ -5662,7 +5662,7 @@
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>R$ 1.050.000,00</t>
+          <t>R$ 589.998,72</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
@@ -5694,22 +5694,22 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>SECRETARIA DE INFRAESTRUTURA URBANA</t>
+          <t>Fundação Municipal de Esportes - Fme</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Pavimentação em pedras irregulares de basalto nas Ruas "A" Trecho II, "B" Trecho III e "H" no Bairro Nossa Senhora Aparecida.</t>
+          <t>Execução de serviços de engenharia para Manutenção Predial e Civil das edificações do município de Indaial e de seus fundos e fundações.</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>J.M.A TERRAPLANAGEM LTDA</t>
+          <t>CONSTRUTORA SCHROEDER E SCHMIDT LTDA</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>43.637.217/0001-10</t>
+          <t>43.887.548/0001-08</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
@@ -5719,12 +5719,12 @@
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>R$ 589.998,72</t>
+          <t>R$ 134.268,71</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>obras_civis</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
@@ -5751,22 +5751,22 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Fundação Municipal de Esportes - Fme</t>
+          <t>Prefeitura Municipal de Catanduvas</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Execução de serviços de engenharia para Manutenção Predial e Civil das edificações do município de Indaial e de seus fundos e fundações.</t>
+          <t>Contratação de empresa especializada para execução de pavimentação nos estacionamentos centrais do Município, com fornecimento de matérias e mão de obra, conforme descritos no projeto, memorial descritivo e termo de referência (Anexo “II”) do presente edital.</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>CONSTRUTORA SCHROEDER E SCHMIDT LTDA</t>
+          <t>R3 PRESTACAO DE SERVICOS LTDA</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>43.887.548/0001-08</t>
+          <t>15.371.451/0001-02</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
@@ -5776,12 +5776,12 @@
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>R$ 134.268,71</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>obras_civis</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
@@ -5808,37 +5808,37 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Prefeitura Municipal de Trombudo Central - SC</t>
+          <t>Secretaria Municipal de Planejamento</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>AQUISIÇÃO DE EQUIPAMENTO DE PINTURA E DEMARCAÇÃO VIÁRIA DO TIPO AIRLESS,  DESTINADO À APLICAÇÃO DE TINTA EM SINALIZAÇÃO HORIZONTAL, CONTEMPLANDO PINTURA DE MEIO-FIO, EIXO DE CENTRO (1 OU 2 FAIXAS), FAIXAS DE PEDESTRES E LOMBADAS, COM CAPACIDADE OPERACIONAL E ESPECIFICAÇÕES TÉCNICAS ADEQUADAS PARA ATENDER AOS PADRÕES DE SEGURANÇA VIÁRIA ESTABELECIDOS PELA LEGISLAÇÃO VIGENTE. O EQUIPAMENTO SERÁ UTILIZADO PELAS EQUIPES MUNICIPAIS NA EXECUÇÃO E MANUTENÇÃO DA SINALIZAÇÃO VIÁRIA DE RUAS E VIAS PÚBL...</t>
+          <t>Contratação de empresa para execução de projeto de construção da obra de pavimentação asfáltica e drenagem da Estrada Geral Fazenda de Dentro (Rua Manoel Mendes), Localidade de Fazenda de Dentro,Biguaçu/SC</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>SD COMERCIAL EQUIPAMENTOS LTDA</t>
+          <t>CONSTRUCOES SCHOROEDER LTDA</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>44.802.526/0001-60</t>
+          <t>10.249.046/0001-00</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>28/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>R$ 34.000,00</t>
+          <t>R$ 1.325.157,30</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>drenagem</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
@@ -5865,32 +5865,32 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Prefeitura Municipal de Catanduvas</t>
+          <t>PREFEITURA MUNICIPAL DE BELA VISTA DO TOLDO - SC</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para execução de pavimentação nos estacionamentos centrais do Município, com fornecimento de matérias e mão de obra, conforme descritos no projeto, memorial descritivo e termo de referência (Anexo “II”) do presente edital.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA EXECUÇÃO DE RECUPERAÇÃO DE PAVIMENTAÇÃO ASFÁLTICA NA RUA AUGUSTO KUCHLER.</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>R3 PRESTACAO DE SERVICOS LTDA</t>
+          <t>EPG ENGENHARIA E CONSTRUCOES LTDA</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>15.371.451/0001-02</t>
+          <t>34.605.142/0001-02</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>28/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 598.403,21</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
@@ -5922,22 +5922,22 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>EMASA - Empresa Municipal de Água e Saneamento de Balneário Camboriú</t>
+          <t>Secretaria de Administração</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>AQUISIÇÃO DE CONJUNTOS MOTOBOMBAS SUBMERSÍVEIS PARA SEREM UTILIZADOS NO SISTEMA DE ESGOTAMENTO SANITÁRIO, NO MUNICÍPIO DE BALNEÁRIO CAMBORIÚ/SC.</t>
+          <t>Contratação de empresa especializada para execução de pavimentação em Piso Intertravado, localizado Rua Emilio Figueiredo, no bairro Itinga no município de Araquari incluindo Drenagem Pluvial e Sinalização, com fornecimento de todos os materiais necessários a execução da obra</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>SULZER PUMPS WASTEWATER BRASIL LTDA</t>
+          <t>BELGA CONSTRUCOES LTDA</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>77.153.260/0013-65</t>
+          <t>81.537.672/0001-32</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
@@ -5947,12 +5947,12 @@
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>R$ 6.454.000,00</t>
+          <t>R$ 370.000,00</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>saneamento</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
@@ -5979,22 +5979,22 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Secretaria Municipal de Planejamento</t>
+          <t>Departamento de Urbanismo</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa para execução de projeto de construção da obra de pavimentação asfáltica e drenagem da Estrada Geral Fazenda de Dentro (Rua Manoel Mendes), Localidade de Fazenda de Dentro,Biguaçu/SC</t>
+          <t>Contratação de empresa especializada em serviços de engenharia necessários à execução de pavimentação rural poliédrica na EMNI 003 e EMNI 023 - Linha Bela Vista da Taquara, processo SCC 00005510/2025.</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>CONSTRUCOES SCHOROEDER LTDA</t>
+          <t>MAGUI TRANSPORTES LTDA</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>10.249.046/0001-00</t>
+          <t>06.865.712/0001-50</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
@@ -6004,7 +6004,7 @@
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>R$ 1.325.157,30</t>
+          <t>R$ 358.000,12</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
@@ -6036,22 +6036,22 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE BELA VISTA DO TOLDO - SC</t>
+          <t>FUNDAÇÃO HOSPITALAR DR JOSÉ ATHANAZIO</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA EXECUÇÃO DE RECUPERAÇÃO DE PAVIMENTAÇÃO ASFÁLTICA NA RUA AUGUSTO KUCHLER.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA EXECUÇÃO DE ADEQUAÇÃO DA INFRAESTRUTURA ELÉTRICA E SUBSTITUIÇÃO DO PADRÃO ELÉTRICO DE ENTRADA ATUAL   - SUBESTAÇÃO 300 KVA DA FUNDAÇÃO HOSPITALAR DR. JOSÉ ATHANÁZIO, COM FORNECIMENTO DE MÃO DE OBRA E MATERIAIS, CONFORME PROJETO BÁSICO</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>EPG ENGENHARIA E CONSTRUCOES LTDA</t>
+          <t>LUMINORTE INSTALACAO, MANUTENCAO E COMERCIO DE MATERIAIS ELETRICOS LTDA</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>34.605.142/0001-02</t>
+          <t>40.627.004/0001-19</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
@@ -6061,17 +6061,17 @@
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>R$ 598.403,21</t>
+          <t>R$ 242.900,00</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>projetos</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_HIGH_CONFIDENCE</t>
+          <t>ENGINEERING_REVIEW</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_HIGH_CONFIDENCE</t>
+          <t>ENGINEERING_REVIEW</t>
         </is>
       </c>
     </row>
@@ -6791,7 +6791,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>live-pack-20260725-032739-85524edc</t>
+          <t>live-pack-20260725-033723-8b07813e</t>
         </is>
       </c>
     </row>
@@ -6815,7 +6815,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7706783a722d7b0a1469aa73b2d2a402b10117ae</t>
+          <t>c3b2495fc7c6ebc40e85f1a118e619a9ab4ef202</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(consulting): freeze client-ready-frozen-rc-v2 with content product_rc_sha
Single regenerate of commercial RC v2 from hardened sector classifier.
product_rc_sha is content-addressed (not git tip) to avoid rebind loops.
C filtered setorialmente; E SUCCESS_ZERO; PENDING_HUMAN for second review.
</commit_message>
<xml_diff>
--- a/artifacts/campaigns/CLIENT-READY-RECURRING-CONSULTING-CYCLE-01/client-ready-frozen-rc-v2/consulting-pack.xlsx
+++ b/artifacts/campaigns/CLIENT-READY-RECURRING-CONSULTING-CYCLE-01/client-ready-frozen-rc-v2/consulting-pack.xlsx
@@ -642,7 +642,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Status RC: PENDING_HUMAN | Pack: live-pack-20260725-033723-8b07813e</t>
+          <t>Status RC: PENDING_HUMAN | Pack: live-pack-20260725-034511-57554b1d</t>
         </is>
       </c>
     </row>
@@ -6791,7 +6791,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>live-pack-20260725-033723-8b07813e</t>
+          <t>live-pack-20260725-034511-57554b1d</t>
         </is>
       </c>
     </row>
@@ -6815,7 +6815,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>c3b2495fc7c6ebc40e85f1a118e619a9ab4ef202</t>
+          <t>df2f45b343fc653175461a692f910c17bb1e4af9</t>
         </is>
       </c>
     </row>

</xml_diff>